<commit_message>
Consolidate literature review table columns and make content concise
Merged Study+Year and Detection+Classification method columns into single
columns, shortened contribution/limitation text for better table readability.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/luaran/hand_created/papers/exports/Literature_Review_Table.xlsx
+++ b/luaran/hand_created/papers/exports/Literature_Review_Table.xlsx
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -137,20 +137,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -523,16 +514,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -552,38 +541,25 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Study</t>
+          <t>Study (Year)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>Method</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Detection
-Method</t>
+          <t>Dataset(s) &amp; Scale</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Classification
-Method</t>
+          <t>Key Contribution</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Dataset(s)
-&amp; Scale</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Key Contribution</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Limitation / Gap</t>
         </is>
@@ -592,253 +568,183 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Arshad et al.
+          <t>Arshad et al. (2022)
 [5]</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>2022</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Det: Morphological segmentation + watershed
+Cls: ResNet50V2</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Morphological segmentation
-+ watershed algorithm</t>
+          <t>IML (345 imgs, 4 P. vivax stages)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>ResNet50V2</t>
+          <t>Introduced IML dataset with bbox annotations; two-stage det-cls pipeline</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>IML Lifecycle
-(345 images, 4 P. vivax stages)</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Introduced IML Lifecycle dataset with bounding box annotations; demonstrated viability of two-stage detection-classification pipeline</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Single species (P. vivax); relatively small dataset; no cross-dataset evaluation; no class imbalance handling</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Loddo et al.
+          <t>Single species; small dataset; no cross-dataset eval; no imbalance handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Loddo et al. (2022)
 [6]</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Not applicable
-(classification only)</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>11 CNNs evaluated
-(best: DenseNet-201)</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>MP-IDB + NIH
-(209 + 27,558 images)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>First deep learning baseline for lifecycle stage classification on MP-IDB; comprehensive comparison of 11 CNN architectures</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Classification only — no detection component; single species (P. falciparum); no end-to-end workflow</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Cls only: 11 CNNs evaluated
+(best: DenseNet-201, Acc 99.40%)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>MP-IDB + NIH (209 + 27,558 imgs)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>First DL baseline on MP-IDB; comprehensive 11 CNN comparison</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>No detection component; single species (P. falciparum); no end-to-end workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Zedda et al.
+          <t>Zedda et al. (2022)
 [7]</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>2022</t>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Det: YOLOv5
+Cls: DarkNet-53 (Acc 96.02%)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>YOLOv5</t>
+          <t>MP-IDB (209 imgs, P. falciparum)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>DarkNet-53</t>
+          <t>First YOLO detection on MP-IDB; single-stage det matches cls-only pipelines</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>MP-IDB
-(209 images)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>First application of YOLO-based object detection on MP-IDB; demonstrated single-stage detectors match classification-only pipelines</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Single dataset (MP-IDB); no class imbalance handling; separate detection and classification models</t>
+          <t>Single dataset; no imbalance handling; separate det and cls models</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Zedda et al.
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Zedda et al. (2023)
 [8]</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>YOLO-PAM
-(YOLOv8 + NAM/CBAM
-attention modules)</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Not specified
-(detection focus)</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>IML + MP-IDB
-(313 + 209 images)</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Introduced attention mechanisms (NAM/CBAM) for malaria detection; reduced parameters by 11M vs baseline YOLOv8 while maintaining accuracy</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Detection only — no classification evaluation; specialized architecture limits reproducibility; no class imbalance handling</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Det+Cls: YOLO-PAM
+(YOLOv8 + NAM/CBAM attention)
+mAP@50: 91.8% IML, 83.6% MP-IDB</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>IML + MP-IDB (522 imgs, 2 species)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Attention mechanisms for malaria det; 11M fewer params vs YOLOv8</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Detection-only eval; specialized arch limits reproducibility; no imbalance handling</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Sukumarran et al.
+          <t>Sukumarran et al. (2024)
 [9]</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>2024</t>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Det: YOLOv4/v5 (mAP@50: 96%)
+Cls: DenseNet-121 (Acc 95.5%)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>YOLOv4 (optimised)
-+ YOLOv5 comparison</t>
+          <t>IML + MP-IDB (522 imgs, 2 species)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>DenseNet-121</t>
+          <t>YOLOv4 vs v5 comparison; two-stage det then species cls</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>IML + MP-IDB
-(313 + 209 images)</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Comparative evaluation of YOLOv4 vs YOLOv5 for malaria detection; two-stage detection then species classification</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Fixed architecture (no multi-model comparison for classification); no class imbalance handling; per-detector training</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="84" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>This study
+          <t>Fixed cls arch (no multi-model comparison); no imbalance handling; per-detector training</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>This study (2025)
 Ours</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>YOLOv10/v11/v12
-Medium (20.1M params)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>6 CNNs: DenseNet121,
-EfficientNet-B0/B1/B2,
-ResNet50/101</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>4 datasets:
-IML (313), MP-IDB Species (209),
-MP-IDB Stages (209), MD-2019 (813)
-Total: 1,544 images</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Shared classification architecture (train-once-reuse); systematic 3-YOLO x 6-CNN multi-model evaluation; Focal Loss for extreme imbalance (up to 54:1); parameter-efficient models (46-89 MB)</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Limited to 4 public datasets (max 813 images); bounding box only (no pixel-level segmentation); laboratory images only (no field validation)</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Det: YOLOv10/v11/v12 (20.1M params)
+Cls: 6 CNNs (DenseNet, EfficientNet, ResNet)</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>4 datasets, 1,544 imgs total
+(IML, MP-IDB Species/Stages, MD-2019)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Shared cls arch (train-once-reuse); 3x6 multi-model eval; Focal Loss for imbalance (up to 54:1); 46-89 MB models</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>4 public datasets (max 813 imgs); bbox only; lab images only</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -851,15 +757,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -879,34 +784,29 @@
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Study</t>
+          <t>Study (Year)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>Key Method</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Key Method</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Gap 1:
 Cross-Dataset
 Robustness</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Gap 2:
 Class Imbalance
 Handling</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Gap 3:
 Computational
@@ -917,34 +817,28 @@
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Arshad et al.
+          <t>Arshad et al. (2022)
 [5]</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Morphological segmentation
-+ ResNet50V2</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Det: Morphological segmentation + watershed</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Single dataset
 (IML only)</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Not addressed
 (standard CE loss)</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Per-detector training
 (no shared architecture)</t>
@@ -952,34 +846,29 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Loddo et al.
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Loddo et al. (2022)
 [6]</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>11 CNNs evaluated</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Cls only: 11 CNNs evaluated</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Single dataset
 (MP-IDB only)</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Not addressed</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Classification only
 (no detection pipeline)</t>
@@ -989,33 +878,27 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Zedda et al.
+          <t>Zedda et al. (2022)
 [7]</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>YOLOv5
-+ DarkNet-53</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Det: YOLOv5</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Single dataset
 (MP-IDB only)</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Not addressed</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Per-detector training
 (separate cls per det)</t>
@@ -1023,34 +906,29 @@
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Zedda et al.
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Zedda et al. (2023)
 [8]</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>YOLO-PAM</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Det+Cls: YOLO-PAM</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>2 datasets
 (IML + MP-IDB)</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Not addressed</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Parameter reduction
 (attention pruning)
@@ -1058,36 +936,30 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Sukumarran et al.
+          <t>Sukumarran et al. (2024)
 [9]</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>2024</t>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Det: YOLOv4/v5 (mAP@50: 96%)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>YOLOv4 (optimised)
-+ DenseNet-121</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>2 datasets
 (IML + MP-IDB)</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Not addressed</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Per-detector training
 (no shared architecture)</t>
@@ -1095,38 +967,32 @@
       </c>
     </row>
     <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>This study
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>This study (2025)
 Ours</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>2025</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Det: YOLOv10/v11/v12 (20.1M params)</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>YOLOv10/v11/v12
-+ 6 CNNs: DenseNet121,</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>4 complementary datasets
 (1,544 total images;
 lifecycle + species + multi-patient)</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Focal Loss (a=1.0, g=1.5)
 + weighted random sampling
 F1: 0.44-1.00 on minorities</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Shared classification
 (train-once-reuse paradigm)
@@ -1137,8 +1003,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>